<commit_message>
fix(UpcomingDebitedCustomerExport): ajust exported customers data including extra stripe informations
</commit_message>
<xml_diff>
--- a/src/test/resources/files/expected_customers_export.xlsx
+++ b/src/test/resources/files/expected_customers_export.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/afryan/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_EE22C379B5496219924AC3B9775F3A4F0472E89B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_C5796372B5496219924AC339EFD8163DE47CC1D4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,36 +20,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+  <si>
+    <t>Stripe Customer ID</t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>Stripe Customer ID</t>
-  </si>
-  <si>
-    <t>Unknown</t>
+    <t>Stripe Name</t>
+  </si>
+  <si>
+    <t>Dashboard Customer Name (Invoice)</t>
+  </si>
+  <si>
+    <t>Creation Datetime</t>
+  </si>
+  <si>
+    <t>Facture générée</t>
+  </si>
+  <si>
+    <t>john-uuid-gen-v4</t>
+  </si>
+  <si>
+    <t>john@example.com</t>
   </si>
   <si>
     <t>John Doe</t>
   </si>
   <si>
-    <t>john@example.com</t>
-  </si>
-  <si>
-    <t>john-uuid-gen-v4</t>
+    <t>2026-01-01T09:00</t>
+  </si>
+  <si>
+    <t>jane-uuid-gen-v4</t>
+  </si>
+  <si>
+    <t>jane@example.com</t>
+  </si>
+  <si>
+    <t>Jane</t>
   </si>
   <si>
     <t>Jane Doe</t>
-  </si>
-  <si>
-    <t>jane@example.com</t>
-  </si>
-  <si>
-    <t>jane-uuid-gen-v4</t>
   </si>
 </sst>
 </file>
@@ -68,7 +80,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -433,16 +444,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -455,33 +468,51 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="b">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="b">
         <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>